<commit_message>
Pie chart and unit bar chart
</commit_message>
<xml_diff>
--- a/data/raw/coffee_preferences.xlsx
+++ b/data/raw/coffee_preferences.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chloe\Downloads\S2 2026\FIT3179\coffee-visualisation\coffee-visualisation\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEBB90EA-C329-4748-8B89-85F75D59926C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32F690FC-4B2C-4788-B908-BE35ADAF4864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14870" yWindow="0" windowWidth="7770" windowHeight="14410" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3120" yWindow="3200" windowWidth="16920" windowHeight="10490" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,10 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
-  <si>
-    <t>Beverage Type</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
   <si>
     <t>Latte</t>
   </si>
@@ -45,29 +42,41 @@
     <t>Espresso</t>
   </si>
   <si>
-    <t>Chai</t>
-  </si>
-  <si>
     <t>Mocha</t>
   </si>
   <si>
-    <t>Hot Chocolate</t>
-  </si>
-  <si>
-    <t>Hot Tea</t>
-  </si>
-  <si>
     <t>Piccolo</t>
   </si>
   <si>
     <t>Percentage Preferences</t>
+  </si>
+  <si>
+    <t>Drink</t>
+  </si>
+  <si>
+    <t>Other Beverages</t>
+  </si>
+  <si>
+    <t>Chocolate</t>
+  </si>
+  <si>
+    <t>Milk</t>
+  </si>
+  <si>
+    <t>Foam</t>
+  </si>
+  <si>
+    <t>Water</t>
+  </si>
+  <si>
+    <t>Total</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -76,6 +85,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -104,9 +121,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -388,96 +411,264 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="16.08984375" customWidth="1"/>
+    <col min="2" max="8" width="12.7265625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3">
+        <v>0.27</v>
+      </c>
+      <c r="C2">
+        <v>30</v>
+      </c>
+      <c r="D2">
+        <v>150</v>
+      </c>
+      <c r="E2">
+        <v>20</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1">
-        <v>0.27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="B3" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="C3">
+        <v>30</v>
+      </c>
+      <c r="D3">
+        <v>160</v>
+      </c>
+      <c r="E3">
+        <v>10</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="1">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="B4" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="C4">
+        <v>30</v>
+      </c>
+      <c r="D4">
+        <v>110</v>
+      </c>
+      <c r="E4">
+        <v>60</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="1">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="B5" s="3">
+        <v>0.08</v>
+      </c>
+      <c r="C5">
+        <v>30</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>170</v>
+      </c>
+      <c r="H5">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="1">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="B6" s="3">
+        <v>0.06</v>
+      </c>
+      <c r="C6">
+        <v>30</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="1">
-        <v>0.06</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+      <c r="B7" s="3">
+        <v>0.03</v>
+      </c>
+      <c r="C7">
+        <v>30</v>
+      </c>
+      <c r="D7">
+        <v>120</v>
+      </c>
+      <c r="E7">
+        <v>20</v>
+      </c>
+      <c r="F7">
+        <v>30</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="1">
-        <v>0.04</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="1">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B8" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="C8">
+        <v>30</v>
+      </c>
+      <c r="D8">
+        <v>60</v>
+      </c>
+      <c r="E8">
+        <v>10</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="1">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="1">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" s="1">
-        <v>0.02</v>
-      </c>
+      <c r="B9" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D14" s="1"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D15" s="1"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D16" s="1"/>
+    </row>
+    <row r="17" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D17" s="1"/>
+    </row>
+    <row r="18" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D18" s="1"/>
+    </row>
+    <row r="19" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D19" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>